<commit_message>
Fix NaN handling in upload_excel function and update data.xlsx
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\.Work\AABS\Qdrant\Context_flow\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBB90A7A-E07A-424A-8E18-407A46B6A563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28C59E92-6583-4F4F-9F9D-29026568E958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,9 +42,6 @@
     <t>Qdrant is a vector database designed for semantic search. It stores embeddings alongside JSON payloads for flexible querying.</t>
   </si>
   <si>
-    <t>https://qdrant.tech/logo.png</t>
-  </si>
-  <si>
     <t>Semantic Chunking</t>
   </si>
   <si>
@@ -64,6 +61,9 @@
   </si>
   <si>
     <t>Excel files can be uploaded and converted into JSON records before being stored in Qdrant.</t>
+  </si>
+  <si>
+    <t>https://qdrant.tech/img/brand-resources-logos/qdrant-brandmark-red.png</t>
   </si>
 </sst>
 </file>
@@ -427,7 +427,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="230.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -435,35 +435,35 @@
         <v>4</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>7</v>
       </c>
       <c r="C3" s="2"/>
     </row>
-    <row r="4" spans="1:3" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="3" t="s">
+    </row>
+    <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="C5" s="2"/>
     </row>
@@ -473,5 +473,6 @@
     <hyperlink ref="C4" r:id="rId2" xr:uid="{6AAA69A4-9303-4812-9C2A-82159FBEE1B5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor: remove unused search functionality and related schema from documents endpoint
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\.Work\AABS\Qdrant\Context_flow\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28C59E92-6583-4F4F-9F9D-29026568E958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F6F2D7-2C8E-477A-8CF0-A4B94F5481EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,9 +54,6 @@
     <t>FastAPI allows you to create fast REST APIs. It integrates well with Qdrant for ML-powered applications.</t>
   </si>
   <si>
-    <t>https://fastapi.tiangolo.com/img/logo-margin/logo-teal.png</t>
-  </si>
-  <si>
     <t>Excel Ingestion</t>
   </si>
   <si>
@@ -64,6 +61,9 @@
   </si>
   <si>
     <t>https://qdrant.tech/img/brand-resources-logos/qdrant-brandmark-red.png</t>
+  </si>
+  <si>
+    <t>https://cdn.worldvectorlogo.com/logos/fastapi.svg</t>
   </si>
 </sst>
 </file>
@@ -435,7 +435,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -455,15 +455,15 @@
         <v>8</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>11</v>
       </c>
       <c r="C5" s="2"/>
     </row>

</xml_diff>